<commit_message>
Update 1. Tracker Spreadsheet.xlsx
</commit_message>
<xml_diff>
--- a/Referances/1. Tracker Spreadsheet.xlsx
+++ b/Referances/1. Tracker Spreadsheet.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frase\OneDrive\Documents\GitHub\Honours-Project-2025\Referances\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2fbaacdcdd0fd4d2/Documents/GitHub/Honours-Project-2025/Referances/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E676E0C-34EB-46CA-B44B-AD541F636144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{8E676E0C-34EB-46CA-B44B-AD541F636144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95ED148D-539A-4C6E-9CE9-B544F30D0D44}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{EC4575A0-A6B1-4C09-B265-56B5475FECA2}"/>
   </bookViews>

</xml_diff>